<commit_message>
Add special insurer medical mapping support
</commit_message>
<xml_diff>
--- a/保全名单.xlsx
+++ b/保全名单.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dongjiajun/Documents/vibe coding/保全时效优化/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D11B748B-5DBC-0F40-8326-E75BA3086306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{383D59B7-96B8-5C4B-AFDB-94AB41464FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="620" windowWidth="51200" windowHeight="28180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1060" yWindow="780" windowWidth="37340" windowHeight="24080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="4" r:id="rId1"/>
@@ -2173,9 +2173,6 @@
     <t>1972-10-20</t>
   </si>
   <si>
-    <t>沈阳</t>
-  </si>
-  <si>
     <t>1994-11-28</t>
   </si>
   <si>
@@ -2980,7 +2977,11 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>中国人民健康保险股份有限公司上海分公司</t>
+    <t>人保健康-LSBLD</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>东莞</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -3549,8 +3550,8 @@
       <c r="V2" t="s">
         <v>55</v>
       </c>
-      <c r="W2" t="s">
-        <v>56</v>
+      <c r="W2" s="4" t="s">
+        <v>981</v>
       </c>
       <c r="X2" t="s">
         <v>40</v>
@@ -3635,8 +3636,8 @@
       <c r="V3" t="s">
         <v>55</v>
       </c>
-      <c r="W3" t="s">
-        <v>56</v>
+      <c r="W3" s="4" t="s">
+        <v>981</v>
       </c>
       <c r="X3" t="s">
         <v>40</v>
@@ -3721,8 +3722,8 @@
       <c r="V4" t="s">
         <v>55</v>
       </c>
-      <c r="W4" t="s">
-        <v>56</v>
+      <c r="W4" s="4" t="s">
+        <v>981</v>
       </c>
       <c r="X4" t="s">
         <v>40</v>
@@ -3774,8 +3775,8 @@
       <c r="K5" t="s">
         <v>32</v>
       </c>
-      <c r="L5" t="s">
-        <v>714</v>
+      <c r="L5" s="4" t="s">
+        <v>982</v>
       </c>
       <c r="M5" t="s">
         <v>49</v>
@@ -3807,8 +3808,8 @@
       <c r="V5" t="s">
         <v>55</v>
       </c>
-      <c r="W5" t="s">
-        <v>56</v>
+      <c r="W5" s="4" t="s">
+        <v>981</v>
       </c>
       <c r="X5" t="s">
         <v>40</v>
@@ -3896,8 +3897,8 @@
       <c r="V6" t="s">
         <v>55</v>
       </c>
-      <c r="W6" t="s">
-        <v>56</v>
+      <c r="W6" s="4" t="s">
+        <v>981</v>
       </c>
       <c r="X6" t="s">
         <v>40</v>
@@ -3982,8 +3983,8 @@
       <c r="V7" t="s">
         <v>55</v>
       </c>
-      <c r="W7" t="s">
-        <v>56</v>
+      <c r="W7" s="4" t="s">
+        <v>981</v>
       </c>
       <c r="X7" t="s">
         <v>40</v>
@@ -4068,8 +4069,8 @@
       <c r="V8" t="s">
         <v>55</v>
       </c>
-      <c r="W8" t="s">
-        <v>56</v>
+      <c r="W8" s="4" t="s">
+        <v>981</v>
       </c>
       <c r="X8" t="s">
         <v>40</v>
@@ -4095,7 +4096,7 @@
         <v>43</v>
       </c>
       <c r="C9" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="D9" t="s">
         <v>31</v>
@@ -4154,8 +4155,8 @@
       <c r="V9" t="s">
         <v>55</v>
       </c>
-      <c r="W9" t="s">
-        <v>56</v>
+      <c r="W9" s="4" t="s">
+        <v>981</v>
       </c>
       <c r="X9" t="s">
         <v>40</v>
@@ -4246,8 +4247,8 @@
       <c r="V10" t="s">
         <v>55</v>
       </c>
-      <c r="W10" t="s">
-        <v>56</v>
+      <c r="W10" s="4" t="s">
+        <v>981</v>
       </c>
       <c r="X10" t="s">
         <v>40</v>
@@ -4332,8 +4333,8 @@
       <c r="V11" t="s">
         <v>55</v>
       </c>
-      <c r="W11" t="s">
-        <v>56</v>
+      <c r="W11" s="4" t="s">
+        <v>981</v>
       </c>
       <c r="X11" t="s">
         <v>40</v>
@@ -4418,8 +4419,8 @@
       <c r="V12" t="s">
         <v>205</v>
       </c>
-      <c r="W12" t="s">
-        <v>56</v>
+      <c r="W12" s="4" t="s">
+        <v>981</v>
       </c>
       <c r="X12" t="s">
         <v>40</v>
@@ -4439,34 +4440,34 @@
     </row>
     <row r="13" spans="1:30">
       <c r="A13" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="B13" t="s">
         <v>43</v>
       </c>
       <c r="C13" t="s">
+        <v>717</v>
+      </c>
+      <c r="D13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" t="s">
         <v>718</v>
       </c>
-      <c r="D13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E13" t="s">
-        <v>719</v>
-      </c>
       <c r="F13" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="G13" t="s">
         <v>43</v>
       </c>
       <c r="H13" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="I13" t="s">
         <v>31</v>
       </c>
       <c r="J13" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="K13" t="s">
         <v>32</v>
@@ -4504,8 +4505,8 @@
       <c r="V13" t="s">
         <v>205</v>
       </c>
-      <c r="W13" t="s">
-        <v>56</v>
+      <c r="W13" s="4" t="s">
+        <v>981</v>
       </c>
       <c r="X13" t="s">
         <v>40</v>
@@ -4587,8 +4588,8 @@
       <c r="V14" t="s">
         <v>205</v>
       </c>
-      <c r="W14" t="s">
-        <v>56</v>
+      <c r="W14" s="4" t="s">
+        <v>981</v>
       </c>
       <c r="X14" t="s">
         <v>40</v>
@@ -4608,34 +4609,34 @@
     </row>
     <row r="15" spans="1:30">
       <c r="A15" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="B15" t="s">
         <v>43</v>
       </c>
       <c r="C15" t="s">
+        <v>731</v>
+      </c>
+      <c r="D15" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15" t="s">
         <v>732</v>
       </c>
-      <c r="D15" t="s">
-        <v>31</v>
-      </c>
-      <c r="E15" t="s">
-        <v>733</v>
-      </c>
       <c r="F15" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="G15" t="s">
         <v>30</v>
       </c>
       <c r="H15" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="I15" t="s">
         <v>31</v>
       </c>
       <c r="J15" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="K15" t="s">
         <v>93</v>
@@ -4670,8 +4671,8 @@
       <c r="V15" t="s">
         <v>205</v>
       </c>
-      <c r="W15" t="s">
-        <v>56</v>
+      <c r="W15" s="4" t="s">
+        <v>981</v>
       </c>
       <c r="X15" t="s">
         <v>40</v>
@@ -4757,7 +4758,7 @@
         <v>210</v>
       </c>
       <c r="W16" s="4" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="X16" t="s">
         <v>40</v>
@@ -4839,8 +4840,8 @@
       <c r="V17" t="s">
         <v>205</v>
       </c>
-      <c r="W17" t="s">
-        <v>56</v>
+      <c r="W17" s="4" t="s">
+        <v>981</v>
       </c>
       <c r="X17" t="s">
         <v>40</v>
@@ -4925,8 +4926,8 @@
       <c r="V18" t="s">
         <v>229</v>
       </c>
-      <c r="W18" t="s">
-        <v>56</v>
+      <c r="W18" s="4" t="s">
+        <v>981</v>
       </c>
       <c r="X18" t="s">
         <v>40</v>
@@ -5011,8 +5012,8 @@
       <c r="V19" t="s">
         <v>277</v>
       </c>
-      <c r="W19" t="s">
-        <v>56</v>
+      <c r="W19" s="4" t="s">
+        <v>981</v>
       </c>
       <c r="X19" t="s">
         <v>40</v>
@@ -5032,34 +5033,34 @@
     </row>
     <row r="20" spans="1:30">
       <c r="A20" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="B20" t="s">
         <v>30</v>
       </c>
       <c r="C20" t="s">
+        <v>734</v>
+      </c>
+      <c r="D20" t="s">
+        <v>31</v>
+      </c>
+      <c r="E20" t="s">
         <v>735</v>
       </c>
-      <c r="D20" t="s">
-        <v>31</v>
-      </c>
-      <c r="E20" t="s">
-        <v>736</v>
-      </c>
       <c r="F20" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="G20" t="s">
         <v>30</v>
       </c>
       <c r="H20" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="I20" t="s">
         <v>31</v>
       </c>
       <c r="J20" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="K20" t="s">
         <v>32</v>
@@ -6233,34 +6234,34 @@
     </row>
     <row r="34" spans="1:30">
       <c r="A34" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="B34" t="s">
         <v>30</v>
       </c>
       <c r="C34" t="s">
+        <v>741</v>
+      </c>
+      <c r="D34" t="s">
+        <v>31</v>
+      </c>
+      <c r="E34" t="s">
         <v>742</v>
       </c>
-      <c r="D34" t="s">
-        <v>31</v>
-      </c>
-      <c r="E34" t="s">
-        <v>743</v>
-      </c>
       <c r="F34" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="G34" t="s">
         <v>30</v>
       </c>
       <c r="H34" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="I34" t="s">
         <v>31</v>
       </c>
       <c r="J34" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="K34" t="s">
         <v>32</v>
@@ -6269,7 +6270,7 @@
         <v>103</v>
       </c>
       <c r="M34" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="N34" t="s">
         <v>301</v>
@@ -6278,7 +6279,7 @@
         <v>36</v>
       </c>
       <c r="P34" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="Q34" t="s">
         <v>105</v>
@@ -6293,10 +6294,10 @@
         <v>139</v>
       </c>
       <c r="U34" t="s">
+        <v>746</v>
+      </c>
+      <c r="V34" t="s">
         <v>747</v>
-      </c>
-      <c r="V34" t="s">
-        <v>748</v>
       </c>
       <c r="W34" t="s">
         <v>56</v>
@@ -6308,7 +6309,7 @@
         <v>301</v>
       </c>
       <c r="AA34" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="AB34" t="s">
         <v>301</v>
@@ -9128,7 +9129,7 @@
         <v>424</v>
       </c>
       <c r="W67" s="4" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="X67" t="s">
         <v>40</v>
@@ -9578,34 +9579,34 @@
     </row>
     <row r="73" spans="1:30">
       <c r="A73" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="B73" t="s">
         <v>30</v>
       </c>
       <c r="C73" t="s">
+        <v>758</v>
+      </c>
+      <c r="D73" t="s">
+        <v>31</v>
+      </c>
+      <c r="E73" t="s">
         <v>759</v>
       </c>
-      <c r="D73" t="s">
-        <v>31</v>
-      </c>
-      <c r="E73" t="s">
-        <v>760</v>
-      </c>
       <c r="F73" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="G73" t="s">
         <v>30</v>
       </c>
       <c r="H73" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="I73" t="s">
         <v>31</v>
       </c>
       <c r="J73" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="K73" t="s">
         <v>32</v>
@@ -9750,34 +9751,34 @@
     </row>
     <row r="75" spans="1:30">
       <c r="A75" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="B75" t="s">
         <v>43</v>
       </c>
       <c r="C75" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="D75" t="s">
         <v>31</v>
       </c>
       <c r="E75" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="F75" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="G75" t="s">
         <v>43</v>
       </c>
       <c r="H75" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="I75" t="s">
         <v>31</v>
       </c>
       <c r="J75" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="K75" t="s">
         <v>32</v>
@@ -10352,34 +10353,34 @@
     </row>
     <row r="82" spans="1:30">
       <c r="A82" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="B82" t="s">
         <v>30</v>
       </c>
       <c r="C82" t="s">
+        <v>762</v>
+      </c>
+      <c r="D82" t="s">
+        <v>31</v>
+      </c>
+      <c r="E82" t="s">
         <v>763</v>
       </c>
-      <c r="D82" t="s">
-        <v>31</v>
-      </c>
-      <c r="E82" t="s">
-        <v>764</v>
-      </c>
       <c r="F82" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G82" t="s">
         <v>30</v>
       </c>
       <c r="H82" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="I82" t="s">
         <v>31</v>
       </c>
       <c r="J82" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="K82" t="s">
         <v>32</v>
@@ -10397,10 +10398,10 @@
         <v>36</v>
       </c>
       <c r="P82" t="s">
+        <v>765</v>
+      </c>
+      <c r="Q82" t="s">
         <v>766</v>
-      </c>
-      <c r="Q82" t="s">
-        <v>767</v>
       </c>
       <c r="R82" t="s">
         <v>37</v>
@@ -10412,13 +10413,13 @@
         <v>39</v>
       </c>
       <c r="U82" t="s">
+        <v>767</v>
+      </c>
+      <c r="V82" t="s">
         <v>768</v>
       </c>
-      <c r="V82" t="s">
-        <v>769</v>
-      </c>
       <c r="W82" s="4" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="X82" t="s">
         <v>40</v>
@@ -10427,7 +10428,7 @@
         <v>35</v>
       </c>
       <c r="AA82" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="AB82" t="s">
         <v>41</v>
@@ -10438,34 +10439,34 @@
     </row>
     <row r="83" spans="1:30">
       <c r="A83" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="B83" t="s">
         <v>30</v>
       </c>
       <c r="C83" t="s">
+        <v>774</v>
+      </c>
+      <c r="D83" t="s">
+        <v>31</v>
+      </c>
+      <c r="E83" t="s">
         <v>775</v>
       </c>
-      <c r="D83" t="s">
-        <v>31</v>
-      </c>
-      <c r="E83" t="s">
-        <v>776</v>
-      </c>
       <c r="F83" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="G83" t="s">
         <v>30</v>
       </c>
       <c r="H83" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="I83" t="s">
         <v>31</v>
       </c>
       <c r="J83" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="K83" t="s">
         <v>32</v>
@@ -10483,10 +10484,10 @@
         <v>36</v>
       </c>
       <c r="P83" t="s">
+        <v>777</v>
+      </c>
+      <c r="Q83" t="s">
         <v>778</v>
-      </c>
-      <c r="Q83" t="s">
-        <v>779</v>
       </c>
       <c r="R83" t="s">
         <v>37</v>
@@ -10498,13 +10499,13 @@
         <v>134</v>
       </c>
       <c r="U83" t="s">
+        <v>779</v>
+      </c>
+      <c r="V83" t="s">
         <v>780</v>
       </c>
-      <c r="V83" t="s">
-        <v>781</v>
-      </c>
       <c r="W83" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X83" t="s">
         <v>40</v>
@@ -10560,7 +10561,7 @@
         <v>103</v>
       </c>
       <c r="M84" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="N84" t="s">
         <v>157</v>
@@ -10569,10 +10570,10 @@
         <v>36</v>
       </c>
       <c r="P84" t="s">
+        <v>782</v>
+      </c>
+      <c r="Q84" t="s">
         <v>783</v>
-      </c>
-      <c r="Q84" t="s">
-        <v>784</v>
       </c>
       <c r="R84" t="s">
         <v>37</v>
@@ -10590,7 +10591,7 @@
         <v>160</v>
       </c>
       <c r="W84" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X84" t="s">
         <v>40</v>
@@ -10610,34 +10611,34 @@
     </row>
     <row r="85" spans="1:30">
       <c r="A85" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="B85" t="s">
         <v>30</v>
       </c>
       <c r="C85" t="s">
+        <v>785</v>
+      </c>
+      <c r="D85" t="s">
+        <v>31</v>
+      </c>
+      <c r="E85" t="s">
         <v>786</v>
       </c>
-      <c r="D85" t="s">
-        <v>31</v>
-      </c>
-      <c r="E85" t="s">
-        <v>787</v>
-      </c>
       <c r="F85" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="G85" t="s">
         <v>30</v>
       </c>
       <c r="H85" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="I85" t="s">
         <v>31</v>
       </c>
       <c r="J85" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="K85" t="s">
         <v>32</v>
@@ -10646,7 +10647,7 @@
         <v>33</v>
       </c>
       <c r="M85" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="N85" t="s">
         <v>117</v>
@@ -10655,10 +10656,10 @@
         <v>36</v>
       </c>
       <c r="P85" t="s">
+        <v>788</v>
+      </c>
+      <c r="Q85" t="s">
         <v>789</v>
-      </c>
-      <c r="Q85" t="s">
-        <v>790</v>
       </c>
       <c r="R85" t="s">
         <v>37</v>
@@ -10670,13 +10671,13 @@
         <v>134</v>
       </c>
       <c r="U85" t="s">
+        <v>790</v>
+      </c>
+      <c r="V85" t="s">
         <v>791</v>
       </c>
-      <c r="V85" t="s">
-        <v>792</v>
-      </c>
       <c r="W85" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X85" t="s">
         <v>40</v>
@@ -10696,34 +10697,34 @@
     </row>
     <row r="86" spans="1:30">
       <c r="A86" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="B86" t="s">
         <v>43</v>
       </c>
       <c r="C86" t="s">
+        <v>721</v>
+      </c>
+      <c r="D86" t="s">
+        <v>31</v>
+      </c>
+      <c r="E86" t="s">
         <v>722</v>
       </c>
-      <c r="D86" t="s">
-        <v>31</v>
-      </c>
-      <c r="E86" t="s">
-        <v>723</v>
-      </c>
       <c r="F86" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="G86" t="s">
         <v>43</v>
       </c>
       <c r="H86" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="I86" t="s">
         <v>31</v>
       </c>
       <c r="J86" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="K86" t="s">
         <v>32</v>
@@ -10744,7 +10745,7 @@
         <v>202</v>
       </c>
       <c r="Q86" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="R86" t="s">
         <v>37</v>
@@ -10762,7 +10763,7 @@
         <v>205</v>
       </c>
       <c r="W86" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X86" t="s">
         <v>40</v>
@@ -10782,34 +10783,34 @@
     </row>
     <row r="87" spans="1:30">
       <c r="A87" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="B87" t="s">
         <v>30</v>
       </c>
       <c r="C87" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="D87" t="s">
         <v>31</v>
       </c>
       <c r="E87" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="F87" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="G87" t="s">
         <v>30</v>
       </c>
       <c r="H87" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="I87" t="s">
         <v>31</v>
       </c>
       <c r="J87" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="K87" t="s">
         <v>32</v>
@@ -10821,16 +10822,16 @@
         <v>104</v>
       </c>
       <c r="N87" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="O87" t="s">
         <v>36</v>
       </c>
       <c r="P87" t="s">
+        <v>805</v>
+      </c>
+      <c r="Q87" t="s">
         <v>806</v>
-      </c>
-      <c r="Q87" t="s">
-        <v>807</v>
       </c>
       <c r="R87" t="s">
         <v>37</v>
@@ -10842,13 +10843,13 @@
         <v>39</v>
       </c>
       <c r="U87" t="s">
+        <v>807</v>
+      </c>
+      <c r="V87" t="s">
         <v>808</v>
       </c>
-      <c r="V87" t="s">
-        <v>809</v>
-      </c>
       <c r="W87" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X87" t="s">
         <v>40</v>
@@ -10857,7 +10858,7 @@
         <v>119</v>
       </c>
       <c r="AA87" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="AB87" t="s">
         <v>119</v>
@@ -10868,34 +10869,34 @@
     </row>
     <row r="88" spans="1:30">
       <c r="A88" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B88" t="s">
         <v>43</v>
       </c>
       <c r="C88" t="s">
+        <v>798</v>
+      </c>
+      <c r="D88" t="s">
+        <v>31</v>
+      </c>
+      <c r="E88" t="s">
         <v>799</v>
       </c>
-      <c r="D88" t="s">
-        <v>31</v>
-      </c>
-      <c r="E88" t="s">
-        <v>800</v>
-      </c>
       <c r="F88" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="G88" t="s">
         <v>43</v>
       </c>
       <c r="H88" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="I88" t="s">
         <v>31</v>
       </c>
       <c r="J88" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="K88" t="s">
         <v>32</v>
@@ -10904,16 +10905,16 @@
         <v>103</v>
       </c>
       <c r="M88" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="N88" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="O88" t="s">
         <v>36</v>
       </c>
       <c r="P88" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="Q88" t="s">
         <v>247</v>
@@ -10928,13 +10929,13 @@
         <v>227</v>
       </c>
       <c r="U88" t="s">
+        <v>794</v>
+      </c>
+      <c r="V88" t="s">
         <v>795</v>
       </c>
-      <c r="V88" t="s">
-        <v>796</v>
-      </c>
       <c r="W88" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X88" t="s">
         <v>40</v>
@@ -10943,7 +10944,7 @@
         <v>119</v>
       </c>
       <c r="AA88" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="AB88" t="s">
         <v>119</v>
@@ -10954,55 +10955,55 @@
     </row>
     <row r="89" spans="1:30">
       <c r="A89" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="B89" t="s">
         <v>30</v>
       </c>
       <c r="C89" t="s">
+        <v>811</v>
+      </c>
+      <c r="D89" t="s">
+        <v>31</v>
+      </c>
+      <c r="E89" t="s">
         <v>812</v>
       </c>
-      <c r="D89" t="s">
-        <v>31</v>
-      </c>
-      <c r="E89" t="s">
-        <v>813</v>
-      </c>
       <c r="F89" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="G89" t="s">
         <v>30</v>
       </c>
       <c r="H89" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="I89" t="s">
         <v>31</v>
       </c>
       <c r="J89" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="K89" t="s">
         <v>32</v>
       </c>
       <c r="L89" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="M89" t="s">
         <v>41</v>
       </c>
       <c r="N89" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="O89" t="s">
         <v>36</v>
       </c>
       <c r="P89" t="s">
+        <v>815</v>
+      </c>
+      <c r="Q89" t="s">
         <v>816</v>
-      </c>
-      <c r="Q89" t="s">
-        <v>817</v>
       </c>
       <c r="R89" t="s">
         <v>37</v>
@@ -11014,13 +11015,13 @@
         <v>267</v>
       </c>
       <c r="U89" t="s">
+        <v>817</v>
+      </c>
+      <c r="V89" t="s">
         <v>818</v>
       </c>
-      <c r="V89" t="s">
-        <v>819</v>
-      </c>
       <c r="W89" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X89" t="s">
         <v>40</v>
@@ -11029,7 +11030,7 @@
         <v>119</v>
       </c>
       <c r="AA89" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="AB89" t="s">
         <v>119</v>
@@ -11040,40 +11041,40 @@
     </row>
     <row r="90" spans="1:30">
       <c r="A90" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="B90" t="s">
         <v>30</v>
       </c>
       <c r="C90" t="s">
+        <v>824</v>
+      </c>
+      <c r="D90" t="s">
+        <v>31</v>
+      </c>
+      <c r="E90" t="s">
         <v>825</v>
       </c>
-      <c r="D90" t="s">
-        <v>31</v>
-      </c>
-      <c r="E90" t="s">
-        <v>826</v>
-      </c>
       <c r="F90" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="G90" t="s">
         <v>30</v>
       </c>
       <c r="H90" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="I90" t="s">
         <v>31</v>
       </c>
       <c r="J90" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="K90" t="s">
         <v>32</v>
       </c>
       <c r="L90" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="M90" t="s">
         <v>41</v>
@@ -11085,10 +11086,10 @@
         <v>36</v>
       </c>
       <c r="P90" t="s">
+        <v>827</v>
+      </c>
+      <c r="Q90" t="s">
         <v>828</v>
-      </c>
-      <c r="Q90" t="s">
-        <v>829</v>
       </c>
       <c r="R90" t="s">
         <v>37</v>
@@ -11100,13 +11101,13 @@
         <v>130</v>
       </c>
       <c r="U90" t="s">
+        <v>822</v>
+      </c>
+      <c r="V90" t="s">
         <v>823</v>
       </c>
-      <c r="V90" t="s">
-        <v>824</v>
-      </c>
       <c r="W90" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X90" t="s">
         <v>40</v>
@@ -11115,7 +11116,7 @@
         <v>119</v>
       </c>
       <c r="AA90" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="AB90" t="s">
         <v>119</v>
@@ -11126,34 +11127,34 @@
     </row>
     <row r="91" spans="1:30">
       <c r="A91" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="B91" t="s">
         <v>30</v>
       </c>
       <c r="C91" t="s">
+        <v>834</v>
+      </c>
+      <c r="D91" t="s">
+        <v>31</v>
+      </c>
+      <c r="E91" t="s">
         <v>835</v>
       </c>
-      <c r="D91" t="s">
-        <v>31</v>
-      </c>
-      <c r="E91" t="s">
-        <v>836</v>
-      </c>
       <c r="F91" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="G91" t="s">
         <v>30</v>
       </c>
       <c r="H91" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="I91" t="s">
         <v>31</v>
       </c>
       <c r="J91" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="K91" t="s">
         <v>32</v>
@@ -11165,16 +11166,16 @@
         <v>119</v>
       </c>
       <c r="N91" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="O91" t="s">
         <v>36</v>
       </c>
       <c r="P91" t="s">
+        <v>837</v>
+      </c>
+      <c r="Q91" t="s">
         <v>838</v>
-      </c>
-      <c r="Q91" t="s">
-        <v>839</v>
       </c>
       <c r="R91" t="s">
         <v>37</v>
@@ -11186,13 +11187,13 @@
         <v>190</v>
       </c>
       <c r="U91" t="s">
+        <v>830</v>
+      </c>
+      <c r="V91" t="s">
         <v>831</v>
       </c>
-      <c r="V91" t="s">
-        <v>832</v>
-      </c>
       <c r="W91" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X91" t="s">
         <v>40</v>
@@ -11201,7 +11202,7 @@
         <v>119</v>
       </c>
       <c r="AA91" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="AB91" t="s">
         <v>119</v>
@@ -11212,43 +11213,43 @@
     </row>
     <row r="92" spans="1:30">
       <c r="A92" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="B92" t="s">
         <v>30</v>
       </c>
       <c r="C92" t="s">
+        <v>840</v>
+      </c>
+      <c r="D92" t="s">
+        <v>31</v>
+      </c>
+      <c r="E92" t="s">
         <v>841</v>
       </c>
-      <c r="D92" t="s">
-        <v>31</v>
-      </c>
-      <c r="E92" t="s">
-        <v>842</v>
-      </c>
       <c r="F92" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="G92" t="s">
         <v>30</v>
       </c>
       <c r="H92" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="I92" t="s">
         <v>31</v>
       </c>
       <c r="J92" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="K92" t="s">
         <v>32</v>
       </c>
       <c r="L92" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="M92" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="N92" t="s">
         <v>314</v>
@@ -11257,10 +11258,10 @@
         <v>36</v>
       </c>
       <c r="P92" t="s">
+        <v>844</v>
+      </c>
+      <c r="Q92" t="s">
         <v>845</v>
-      </c>
-      <c r="Q92" t="s">
-        <v>846</v>
       </c>
       <c r="R92" t="s">
         <v>37</v>
@@ -11278,7 +11279,7 @@
         <v>316</v>
       </c>
       <c r="W92" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X92" t="s">
         <v>40</v>
@@ -11298,7 +11299,7 @@
     </row>
     <row r="93" spans="1:30">
       <c r="A93" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="B93" t="s">
         <v>30</v>
@@ -11310,28 +11311,28 @@
         <v>31</v>
       </c>
       <c r="E93" t="s">
+        <v>847</v>
+      </c>
+      <c r="F93" t="s">
         <v>848</v>
-      </c>
-      <c r="F93" t="s">
-        <v>849</v>
       </c>
       <c r="G93" t="s">
         <v>43</v>
       </c>
       <c r="H93" t="s">
+        <v>849</v>
+      </c>
+      <c r="I93" t="s">
+        <v>31</v>
+      </c>
+      <c r="J93" t="s">
         <v>850</v>
-      </c>
-      <c r="I93" t="s">
-        <v>31</v>
-      </c>
-      <c r="J93" t="s">
-        <v>851</v>
       </c>
       <c r="K93" t="s">
         <v>93</v>
       </c>
       <c r="M93" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="N93" t="s">
         <v>314</v>
@@ -11340,28 +11341,28 @@
         <v>36</v>
       </c>
       <c r="P93" t="s">
+        <v>852</v>
+      </c>
+      <c r="Q93" t="s">
         <v>853</v>
       </c>
-      <c r="Q93" t="s">
+      <c r="R93" t="s">
+        <v>37</v>
+      </c>
+      <c r="S93" t="s">
         <v>854</v>
-      </c>
-      <c r="R93" t="s">
-        <v>37</v>
-      </c>
-      <c r="S93" t="s">
-        <v>855</v>
       </c>
       <c r="T93" t="s">
         <v>107</v>
       </c>
       <c r="U93" t="s">
+        <v>855</v>
+      </c>
+      <c r="V93" t="s">
         <v>856</v>
       </c>
-      <c r="V93" t="s">
-        <v>857</v>
-      </c>
       <c r="W93" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X93" t="s">
         <v>40</v>
@@ -11370,7 +11371,7 @@
         <v>301</v>
       </c>
       <c r="AA93" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="AB93" t="s">
         <v>301</v>
@@ -11381,34 +11382,34 @@
     </row>
     <row r="94" spans="1:30">
       <c r="A94" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="B94" t="s">
         <v>30</v>
       </c>
       <c r="C94" t="s">
+        <v>862</v>
+      </c>
+      <c r="D94" t="s">
+        <v>31</v>
+      </c>
+      <c r="E94" t="s">
         <v>863</v>
       </c>
-      <c r="D94" t="s">
-        <v>31</v>
-      </c>
-      <c r="E94" t="s">
-        <v>864</v>
-      </c>
       <c r="F94" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="G94" t="s">
         <v>30</v>
       </c>
       <c r="H94" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="I94" t="s">
         <v>31</v>
       </c>
       <c r="J94" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="K94" t="s">
         <v>32</v>
@@ -11426,28 +11427,28 @@
         <v>36</v>
       </c>
       <c r="P94" t="s">
+        <v>865</v>
+      </c>
+      <c r="Q94" t="s">
         <v>866</v>
       </c>
-      <c r="Q94" t="s">
-        <v>867</v>
-      </c>
       <c r="R94" t="s">
         <v>37</v>
       </c>
       <c r="S94" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="T94" t="s">
         <v>237</v>
       </c>
       <c r="U94" t="s">
+        <v>867</v>
+      </c>
+      <c r="V94" t="s">
         <v>868</v>
       </c>
-      <c r="V94" t="s">
-        <v>869</v>
-      </c>
       <c r="W94" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X94" t="s">
         <v>40</v>
@@ -11456,7 +11457,7 @@
         <v>417</v>
       </c>
       <c r="AA94" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="AB94" t="s">
         <v>417</v>
@@ -11467,40 +11468,40 @@
     </row>
     <row r="95" spans="1:30">
       <c r="A95" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="B95" t="s">
         <v>30</v>
       </c>
       <c r="C95" t="s">
+        <v>870</v>
+      </c>
+      <c r="D95" t="s">
+        <v>31</v>
+      </c>
+      <c r="E95" t="s">
         <v>871</v>
       </c>
-      <c r="D95" t="s">
-        <v>31</v>
-      </c>
-      <c r="E95" t="s">
-        <v>872</v>
-      </c>
       <c r="F95" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="G95" t="s">
         <v>30</v>
       </c>
       <c r="H95" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="I95" t="s">
         <v>31</v>
       </c>
       <c r="J95" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="K95" t="s">
         <v>32</v>
       </c>
       <c r="L95" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="M95" t="s">
         <v>149</v>
@@ -11512,10 +11513,10 @@
         <v>36</v>
       </c>
       <c r="P95" t="s">
+        <v>874</v>
+      </c>
+      <c r="Q95" t="s">
         <v>875</v>
-      </c>
-      <c r="Q95" t="s">
-        <v>876</v>
       </c>
       <c r="R95" t="s">
         <v>37</v>
@@ -11527,13 +11528,13 @@
         <v>126</v>
       </c>
       <c r="U95" t="s">
+        <v>876</v>
+      </c>
+      <c r="V95" t="s">
         <v>877</v>
       </c>
-      <c r="V95" t="s">
-        <v>878</v>
-      </c>
       <c r="W95" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X95" t="s">
         <v>40</v>
@@ -11542,7 +11543,7 @@
         <v>417</v>
       </c>
       <c r="AA95" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="AB95" t="s">
         <v>417</v>
@@ -11553,34 +11554,34 @@
     </row>
     <row r="96" spans="1:30">
       <c r="A96" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B96" t="s">
         <v>30</v>
       </c>
       <c r="C96" t="s">
+        <v>880</v>
+      </c>
+      <c r="D96" t="s">
+        <v>31</v>
+      </c>
+      <c r="E96" t="s">
         <v>881</v>
       </c>
-      <c r="D96" t="s">
-        <v>31</v>
-      </c>
-      <c r="E96" t="s">
-        <v>882</v>
-      </c>
       <c r="F96" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="G96" t="s">
         <v>30</v>
       </c>
       <c r="H96" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="I96" t="s">
         <v>31</v>
       </c>
       <c r="J96" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="K96" t="s">
         <v>32</v>
@@ -11589,7 +11590,7 @@
         <v>125</v>
       </c>
       <c r="M96" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="N96" t="s">
         <v>35</v>
@@ -11598,10 +11599,10 @@
         <v>36</v>
       </c>
       <c r="P96" t="s">
+        <v>884</v>
+      </c>
+      <c r="Q96" t="s">
         <v>885</v>
-      </c>
-      <c r="Q96" t="s">
-        <v>886</v>
       </c>
       <c r="R96" t="s">
         <v>37</v>
@@ -11613,13 +11614,13 @@
         <v>126</v>
       </c>
       <c r="U96" t="s">
+        <v>886</v>
+      </c>
+      <c r="V96" t="s">
         <v>887</v>
       </c>
-      <c r="V96" t="s">
-        <v>888</v>
-      </c>
       <c r="W96" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X96" t="s">
         <v>40</v>
@@ -11628,7 +11629,7 @@
         <v>417</v>
       </c>
       <c r="AA96" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="AB96" t="s">
         <v>417</v>
@@ -11639,34 +11640,34 @@
     </row>
     <row r="97" spans="1:30">
       <c r="A97" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="B97" t="s">
         <v>43</v>
       </c>
       <c r="C97" t="s">
+        <v>897</v>
+      </c>
+      <c r="D97" t="s">
+        <v>31</v>
+      </c>
+      <c r="E97" t="s">
         <v>898</v>
       </c>
-      <c r="D97" t="s">
-        <v>31</v>
-      </c>
-      <c r="E97" t="s">
-        <v>899</v>
-      </c>
       <c r="F97" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="G97" t="s">
         <v>30</v>
       </c>
       <c r="H97" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="I97" t="s">
         <v>31</v>
       </c>
       <c r="J97" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="K97" t="s">
         <v>93</v>
@@ -11681,7 +11682,7 @@
         <v>36</v>
       </c>
       <c r="P97" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="Q97" t="s">
         <v>269</v>
@@ -11696,13 +11697,13 @@
         <v>134</v>
       </c>
       <c r="U97" t="s">
+        <v>893</v>
+      </c>
+      <c r="V97" t="s">
         <v>894</v>
       </c>
-      <c r="V97" t="s">
-        <v>895</v>
-      </c>
       <c r="W97" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X97" t="s">
         <v>40</v>
@@ -11711,7 +11712,7 @@
         <v>417</v>
       </c>
       <c r="AA97" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="AB97" t="s">
         <v>417</v>
@@ -11722,34 +11723,34 @@
     </row>
     <row r="98" spans="1:30">
       <c r="A98" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="B98" t="s">
         <v>30</v>
       </c>
       <c r="C98" t="s">
+        <v>900</v>
+      </c>
+      <c r="D98" t="s">
+        <v>31</v>
+      </c>
+      <c r="E98" t="s">
         <v>901</v>
       </c>
-      <c r="D98" t="s">
-        <v>31</v>
-      </c>
-      <c r="E98" t="s">
-        <v>902</v>
-      </c>
       <c r="F98" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G98" t="s">
         <v>30</v>
       </c>
       <c r="H98" t="s">
+        <v>902</v>
+      </c>
+      <c r="I98" t="s">
+        <v>31</v>
+      </c>
+      <c r="J98" t="s">
         <v>903</v>
-      </c>
-      <c r="I98" t="s">
-        <v>31</v>
-      </c>
-      <c r="J98" t="s">
-        <v>904</v>
       </c>
       <c r="K98" t="s">
         <v>93</v>
@@ -11758,7 +11759,7 @@
         <v>94</v>
       </c>
       <c r="M98" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="N98" t="s">
         <v>35</v>
@@ -11767,10 +11768,10 @@
         <v>36</v>
       </c>
       <c r="P98" t="s">
+        <v>905</v>
+      </c>
+      <c r="Q98" t="s">
         <v>906</v>
-      </c>
-      <c r="Q98" t="s">
-        <v>907</v>
       </c>
       <c r="R98" t="s">
         <v>37</v>
@@ -11782,13 +11783,13 @@
         <v>130</v>
       </c>
       <c r="U98" t="s">
+        <v>907</v>
+      </c>
+      <c r="V98" t="s">
         <v>908</v>
       </c>
-      <c r="V98" t="s">
-        <v>909</v>
-      </c>
       <c r="W98" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X98" t="s">
         <v>40</v>
@@ -11797,7 +11798,7 @@
         <v>417</v>
       </c>
       <c r="AA98" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="AB98" t="s">
         <v>417</v>
@@ -11808,34 +11809,34 @@
     </row>
     <row r="99" spans="1:30">
       <c r="A99" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="B99" t="s">
         <v>30</v>
       </c>
       <c r="C99" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="D99" t="s">
         <v>31</v>
       </c>
       <c r="E99" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="F99" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G99" t="s">
         <v>30</v>
       </c>
       <c r="H99" t="s">
+        <v>902</v>
+      </c>
+      <c r="I99" t="s">
+        <v>31</v>
+      </c>
+      <c r="J99" t="s">
         <v>903</v>
-      </c>
-      <c r="I99" t="s">
-        <v>31</v>
-      </c>
-      <c r="J99" t="s">
-        <v>904</v>
       </c>
       <c r="K99" t="s">
         <v>32</v>
@@ -11844,7 +11845,7 @@
         <v>103</v>
       </c>
       <c r="M99" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="N99" t="s">
         <v>35</v>
@@ -11853,10 +11854,10 @@
         <v>36</v>
       </c>
       <c r="P99" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="Q99" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="R99" t="s">
         <v>37</v>
@@ -11868,13 +11869,13 @@
         <v>130</v>
       </c>
       <c r="U99" t="s">
+        <v>907</v>
+      </c>
+      <c r="V99" t="s">
         <v>908</v>
       </c>
-      <c r="V99" t="s">
-        <v>909</v>
-      </c>
       <c r="W99" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X99" t="s">
         <v>40</v>
@@ -11883,7 +11884,7 @@
         <v>417</v>
       </c>
       <c r="AA99" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="AB99" t="s">
         <v>417</v>
@@ -11894,34 +11895,34 @@
     </row>
     <row r="100" spans="1:30">
       <c r="A100" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="B100" t="s">
         <v>30</v>
       </c>
       <c r="C100" t="s">
+        <v>913</v>
+      </c>
+      <c r="D100" t="s">
+        <v>31</v>
+      </c>
+      <c r="E100" t="s">
         <v>914</v>
       </c>
-      <c r="D100" t="s">
-        <v>31</v>
-      </c>
-      <c r="E100" t="s">
-        <v>915</v>
-      </c>
       <c r="F100" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="G100" t="s">
         <v>30</v>
       </c>
       <c r="H100" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="I100" t="s">
         <v>31</v>
       </c>
       <c r="J100" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="K100" t="s">
         <v>32</v>
@@ -11939,10 +11940,10 @@
         <v>36</v>
       </c>
       <c r="P100" t="s">
+        <v>916</v>
+      </c>
+      <c r="Q100" t="s">
         <v>917</v>
-      </c>
-      <c r="Q100" t="s">
-        <v>918</v>
       </c>
       <c r="R100" t="s">
         <v>37</v>
@@ -11954,13 +11955,13 @@
         <v>227</v>
       </c>
       <c r="U100" t="s">
+        <v>918</v>
+      </c>
+      <c r="V100" t="s">
         <v>919</v>
       </c>
-      <c r="V100" t="s">
-        <v>920</v>
-      </c>
       <c r="W100" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X100" t="s">
         <v>40</v>
@@ -11969,7 +11970,7 @@
         <v>410</v>
       </c>
       <c r="AA100" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="AB100" t="s">
         <v>410</v>
@@ -11980,34 +11981,34 @@
     </row>
     <row r="101" spans="1:30">
       <c r="A101" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="B101" t="s">
         <v>43</v>
       </c>
       <c r="C101" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="D101" t="s">
         <v>31</v>
       </c>
       <c r="E101" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="F101" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="G101" t="s">
         <v>43</v>
       </c>
       <c r="H101" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="I101" t="s">
         <v>31</v>
       </c>
       <c r="J101" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="K101" t="s">
         <v>32</v>
@@ -12025,10 +12026,10 @@
         <v>36</v>
       </c>
       <c r="P101" t="s">
+        <v>925</v>
+      </c>
+      <c r="Q101" t="s">
         <v>926</v>
-      </c>
-      <c r="Q101" t="s">
-        <v>927</v>
       </c>
       <c r="R101" t="s">
         <v>37</v>
@@ -12040,13 +12041,13 @@
         <v>267</v>
       </c>
       <c r="U101" t="s">
+        <v>921</v>
+      </c>
+      <c r="V101" t="s">
         <v>922</v>
       </c>
-      <c r="V101" t="s">
-        <v>923</v>
-      </c>
       <c r="W101" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X101" t="s">
         <v>40</v>
@@ -12066,40 +12067,40 @@
     </row>
     <row r="102" spans="1:30">
       <c r="A102" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="B102" t="s">
         <v>30</v>
       </c>
       <c r="C102" t="s">
+        <v>928</v>
+      </c>
+      <c r="D102" t="s">
+        <v>31</v>
+      </c>
+      <c r="E102" t="s">
         <v>929</v>
       </c>
-      <c r="D102" t="s">
-        <v>31</v>
-      </c>
-      <c r="E102" t="s">
-        <v>930</v>
-      </c>
       <c r="F102" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="G102" t="s">
         <v>30</v>
       </c>
       <c r="H102" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="I102" t="s">
         <v>31</v>
       </c>
       <c r="J102" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="K102" t="s">
         <v>32</v>
       </c>
       <c r="L102" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="M102" t="s">
         <v>104</v>
@@ -12111,34 +12112,34 @@
         <v>36</v>
       </c>
       <c r="P102" t="s">
+        <v>932</v>
+      </c>
+      <c r="Q102" t="s">
         <v>933</v>
       </c>
-      <c r="Q102" t="s">
-        <v>934</v>
-      </c>
       <c r="R102" t="s">
         <v>37</v>
       </c>
       <c r="S102" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="T102" t="s">
         <v>134</v>
       </c>
       <c r="U102" t="s">
+        <v>934</v>
+      </c>
+      <c r="V102" t="s">
         <v>935</v>
       </c>
-      <c r="V102" t="s">
-        <v>936</v>
-      </c>
       <c r="W102" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X102" t="s">
         <v>40</v>
       </c>
       <c r="Z102" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="AA102" t="s">
         <v>135</v>
@@ -12152,40 +12153,40 @@
     </row>
     <row r="103" spans="1:30">
       <c r="A103" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="B103" t="s">
         <v>30</v>
       </c>
       <c r="C103" t="s">
+        <v>938</v>
+      </c>
+      <c r="D103" t="s">
+        <v>31</v>
+      </c>
+      <c r="E103" t="s">
         <v>939</v>
       </c>
-      <c r="D103" t="s">
-        <v>31</v>
-      </c>
-      <c r="E103" t="s">
-        <v>940</v>
-      </c>
       <c r="F103" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="G103" t="s">
         <v>30</v>
       </c>
       <c r="H103" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="I103" t="s">
         <v>31</v>
       </c>
       <c r="J103" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="K103" t="s">
         <v>32</v>
       </c>
       <c r="L103" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="M103" t="s">
         <v>44</v>
@@ -12197,10 +12198,10 @@
         <v>36</v>
       </c>
       <c r="P103" t="s">
+        <v>942</v>
+      </c>
+      <c r="Q103" t="s">
         <v>943</v>
-      </c>
-      <c r="Q103" t="s">
-        <v>944</v>
       </c>
       <c r="R103" t="s">
         <v>37</v>
@@ -12212,13 +12213,13 @@
         <v>134</v>
       </c>
       <c r="U103" t="s">
+        <v>944</v>
+      </c>
+      <c r="V103" t="s">
         <v>945</v>
       </c>
-      <c r="V103" t="s">
-        <v>946</v>
-      </c>
       <c r="W103" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X103" t="s">
         <v>40</v>
@@ -12238,40 +12239,40 @@
     </row>
     <row r="104" spans="1:30">
       <c r="A104" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="B104" t="s">
         <v>30</v>
       </c>
       <c r="C104" t="s">
+        <v>947</v>
+      </c>
+      <c r="D104" t="s">
+        <v>31</v>
+      </c>
+      <c r="E104" t="s">
         <v>948</v>
       </c>
-      <c r="D104" t="s">
-        <v>31</v>
-      </c>
-      <c r="E104" t="s">
-        <v>949</v>
-      </c>
       <c r="F104" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="G104" t="s">
         <v>30</v>
       </c>
       <c r="H104" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="I104" t="s">
         <v>31</v>
       </c>
       <c r="J104" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="K104" t="s">
         <v>32</v>
       </c>
       <c r="L104" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="M104" t="s">
         <v>41</v>
@@ -12283,10 +12284,10 @@
         <v>36</v>
       </c>
       <c r="P104" t="s">
+        <v>951</v>
+      </c>
+      <c r="Q104" t="s">
         <v>952</v>
-      </c>
-      <c r="Q104" t="s">
-        <v>953</v>
       </c>
       <c r="R104" t="s">
         <v>37</v>
@@ -12298,13 +12299,13 @@
         <v>126</v>
       </c>
       <c r="U104" t="s">
+        <v>953</v>
+      </c>
+      <c r="V104" t="s">
         <v>954</v>
       </c>
-      <c r="V104" t="s">
-        <v>955</v>
-      </c>
       <c r="W104" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X104" t="s">
         <v>40</v>
@@ -12313,7 +12314,7 @@
         <v>546</v>
       </c>
       <c r="AA104" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="AB104" t="s">
         <v>546</v>
@@ -12324,34 +12325,34 @@
     </row>
     <row r="105" spans="1:30">
       <c r="A105" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="B105" t="s">
         <v>43</v>
       </c>
       <c r="C105" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="D105" t="s">
         <v>31</v>
       </c>
       <c r="E105" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="F105" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="G105" t="s">
         <v>43</v>
       </c>
       <c r="H105" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="I105" t="s">
         <v>31</v>
       </c>
       <c r="J105" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="K105" t="s">
         <v>32</v>
@@ -12363,16 +12364,16 @@
         <v>57</v>
       </c>
       <c r="N105" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="O105" t="s">
         <v>36</v>
       </c>
       <c r="P105" t="s">
+        <v>962</v>
+      </c>
+      <c r="Q105" t="s">
         <v>963</v>
-      </c>
-      <c r="Q105" t="s">
-        <v>964</v>
       </c>
       <c r="R105" t="s">
         <v>37</v>
@@ -12384,13 +12385,13 @@
         <v>268</v>
       </c>
       <c r="U105" t="s">
+        <v>956</v>
+      </c>
+      <c r="V105" t="s">
         <v>957</v>
       </c>
-      <c r="V105" t="s">
-        <v>958</v>
-      </c>
       <c r="W105" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="X105" t="s">
         <v>40</v>
@@ -12399,7 +12400,7 @@
         <v>659</v>
       </c>
       <c r="AA105" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="AB105" t="s">
         <v>659</v>
@@ -12410,34 +12411,34 @@
     </row>
     <row r="106" spans="1:30">
       <c r="A106" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="B106" t="s">
         <v>43</v>
       </c>
       <c r="C106" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="D106" t="s">
         <v>31</v>
       </c>
       <c r="E106" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="F106" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="G106" t="s">
         <v>43</v>
       </c>
       <c r="H106" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="I106" t="s">
         <v>31</v>
       </c>
       <c r="J106" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="K106" t="s">
         <v>32</v>
@@ -12476,7 +12477,7 @@
         <v>176</v>
       </c>
       <c r="W106" s="4" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="X106" t="s">
         <v>40</v>
@@ -12496,34 +12497,34 @@
     </row>
     <row r="107" spans="1:30">
       <c r="A107" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="B107" t="s">
         <v>30</v>
       </c>
       <c r="C107" t="s">
+        <v>969</v>
+      </c>
+      <c r="D107" t="s">
+        <v>31</v>
+      </c>
+      <c r="E107" t="s">
         <v>970</v>
       </c>
-      <c r="D107" t="s">
-        <v>31</v>
-      </c>
-      <c r="E107" t="s">
-        <v>971</v>
-      </c>
       <c r="F107" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="G107" t="s">
         <v>30</v>
       </c>
       <c r="H107" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="I107" t="s">
         <v>31</v>
       </c>
       <c r="J107" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="K107" t="s">
         <v>32</v>
@@ -12535,13 +12536,13 @@
         <v>41</v>
       </c>
       <c r="N107" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="O107" t="s">
         <v>36</v>
       </c>
       <c r="P107" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="Q107" t="s">
         <v>148</v>
@@ -12926,34 +12927,34 @@
     </row>
     <row r="112" spans="1:30">
       <c r="A112" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="B112" t="s">
         <v>43</v>
       </c>
       <c r="C112" t="s">
+        <v>976</v>
+      </c>
+      <c r="D112" t="s">
+        <v>31</v>
+      </c>
+      <c r="E112" t="s">
         <v>977</v>
       </c>
-      <c r="D112" t="s">
-        <v>31</v>
-      </c>
-      <c r="E112" t="s">
-        <v>978</v>
-      </c>
       <c r="F112" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="G112" t="s">
         <v>30</v>
       </c>
       <c r="H112" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="I112" t="s">
         <v>31</v>
       </c>
       <c r="J112" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="K112" t="s">
         <v>93</v>

</xml_diff>